<commit_message>
adv Oled eSpark and Client BOM Tft Link added
</commit_message>
<xml_diff>
--- a/Design Files/Adv-OLED-v2.0/BOM/Client_BOM_OLED-v2.0.xlsx
+++ b/Design Files/Adv-OLED-v2.0/BOM/Client_BOM_OLED-v2.0.xlsx
@@ -12,14 +12,14 @@
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="88">
   <si>
     <t>Component list</t>
   </si>
@@ -271,6 +271,18 @@
   </si>
   <si>
     <t xml:space="preserve">JUSHUO </t>
+  </si>
+  <si>
+    <t>Quantity 5 Board</t>
+  </si>
+  <si>
+    <t>2.4-inch tft LCD display SPI serial port color ST7789ILI9341 4IO port can be driven</t>
+  </si>
+  <si>
+    <t>ST7789ILI9341</t>
+  </si>
+  <si>
+    <t>Reference Link</t>
   </si>
 </sst>
 </file>
@@ -280,7 +292,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -415,6 +427,14 @@
       <strike/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -681,10 +701,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -845,6 +866,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -854,11 +878,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -884,13 +910,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>19942</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>1905000</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
@@ -1198,7 +1224,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1211,10 +1237,12 @@
     <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.42578125" customWidth="1"/>
+    <col min="12" max="12" width="18.28515625" customWidth="1"/>
+    <col min="13" max="13" width="29.42578125" customWidth="1"/>
+    <col min="15" max="15" width="25.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1224,11 +1252,12 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="62"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-    </row>
-    <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+    </row>
+    <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="40"/>
@@ -1244,9 +1273,10 @@
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="38"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L2" s="3"/>
+      <c r="M2" s="38"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="41"/>
@@ -1262,9 +1292,10 @@
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="63"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L3" s="4"/>
+      <c r="M3" s="64"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="41"/>
@@ -1280,9 +1311,10 @@
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="64"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L4" s="66"/>
+      <c r="M4" s="65"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="41"/>
@@ -1298,9 +1330,10 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="64"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L5" s="66"/>
+      <c r="M5" s="65"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="42"/>
@@ -1312,9 +1345,10 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="64"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L6" s="66"/>
+      <c r="M6" s="65"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="43"/>
@@ -1326,9 +1360,10 @@
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="64"/>
-    </row>
-    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L7" s="7"/>
+      <c r="M7" s="65"/>
+    </row>
+    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="44"/>
@@ -1340,9 +1375,10 @@
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="64"/>
-    </row>
-    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L8" s="7"/>
+      <c r="M8" s="65"/>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -1375,10 +1411,13 @@
         <v>47</v>
       </c>
       <c r="L9" s="29" t="s">
+        <v>84</v>
+      </c>
+      <c r="M9" s="29" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="53">
         <f t="shared" ref="B10:B20" si="0">ROW(B10) - ROW($B$9)</f>
@@ -1411,9 +1450,13 @@
       <c r="K10" s="37">
         <v>4</v>
       </c>
-      <c r="L10" s="36"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L10" s="36">
+        <f>K10*5</f>
+        <v>20</v>
+      </c>
+      <c r="M10" s="36"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="51">
         <f>ROW(B11) - ROW($B$9)</f>
@@ -1446,9 +1489,13 @@
       <c r="K11" s="36">
         <v>1</v>
       </c>
-      <c r="L11" s="37"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L11" s="36">
+        <f t="shared" ref="L11:L22" si="1">K11*5</f>
+        <v>5</v>
+      </c>
+      <c r="M11" s="37"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="53">
         <f t="shared" si="0"/>
@@ -1481,9 +1528,13 @@
       <c r="K12" s="55">
         <v>1</v>
       </c>
-      <c r="L12" s="36"/>
-    </row>
-    <row r="13" spans="1:12" ht="48" x14ac:dyDescent="0.25">
+      <c r="L12" s="36">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="M12" s="36"/>
+    </row>
+    <row r="13" spans="1:13" ht="48" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="53">
         <f t="shared" si="0"/>
@@ -1516,9 +1567,13 @@
       <c r="K13" s="37">
         <v>2</v>
       </c>
-      <c r="L13" s="37"/>
-    </row>
-    <row r="14" spans="1:12" ht="24" x14ac:dyDescent="0.25">
+      <c r="L13" s="36">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="M13" s="37"/>
+    </row>
+    <row r="14" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="53">
         <f t="shared" si="0"/>
@@ -1551,9 +1606,13 @@
       <c r="K14" s="37">
         <v>1</v>
       </c>
-      <c r="L14" s="36"/>
-    </row>
-    <row r="15" spans="1:12" ht="36" x14ac:dyDescent="0.25">
+      <c r="L14" s="36">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="M14" s="36"/>
+    </row>
+    <row r="15" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="53">
         <f t="shared" si="0"/>
@@ -1586,9 +1645,13 @@
       <c r="K15" s="37">
         <v>1</v>
       </c>
-      <c r="L15" s="37"/>
-    </row>
-    <row r="16" spans="1:12" ht="24" x14ac:dyDescent="0.25">
+      <c r="L15" s="36">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="M15" s="37"/>
+    </row>
+    <row r="16" spans="1:13" ht="24" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="51">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -1621,12 +1684,16 @@
       <c r="K16" s="36">
         <v>1</v>
       </c>
-      <c r="L16" s="36"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L16" s="36">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="M16" s="36"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="53">
-        <f t="shared" ref="B17" si="1">ROW(B17) - ROW($B$9)</f>
+        <f t="shared" ref="B17" si="2">ROW(B17) - ROW($B$9)</f>
         <v>8</v>
       </c>
       <c r="C17" s="52" t="s">
@@ -1656,9 +1723,13 @@
       <c r="K17" s="37">
         <v>3</v>
       </c>
-      <c r="L17" s="37"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L17" s="36">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="M17" s="37"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
       <c r="B18" s="51">
         <f>ROW(B18) - ROW($B$9)</f>
@@ -1691,12 +1762,16 @@
       <c r="K18" s="36">
         <v>1</v>
       </c>
-      <c r="L18" s="36"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L18" s="36">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="M18" s="36"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="1"/>
       <c r="B19" s="53">
-        <f t="shared" ref="B19" si="2">ROW(B19) - ROW($B$9)</f>
+        <f t="shared" ref="B19" si="3">ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
       <c r="C19" s="54" t="s">
@@ -1726,9 +1801,13 @@
       <c r="K19" s="37">
         <v>4</v>
       </c>
-      <c r="L19" s="37"/>
-    </row>
-    <row r="20" spans="1:12" ht="36" x14ac:dyDescent="0.25">
+      <c r="L19" s="36">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="M19" s="37"/>
+    </row>
+    <row r="20" spans="1:13" ht="36" x14ac:dyDescent="0.25">
       <c r="A20" s="1"/>
       <c r="B20" s="56">
         <f t="shared" si="0"/>
@@ -1759,9 +1838,13 @@
       <c r="K20" s="58">
         <v>3</v>
       </c>
-      <c r="L20" s="59"/>
-    </row>
-    <row r="21" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L20" s="36">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="M20" s="59"/>
+    </row>
+    <row r="21" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="53">
         <v>12</v>
@@ -1793,43 +1876,92 @@
       <c r="K21" s="37">
         <v>1</v>
       </c>
-      <c r="L21" s="65"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L21" s="36">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="M21" s="62"/>
+    </row>
+    <row r="22" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="B22" s="31"/>
-      <c r="C22" s="45"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="35"/>
-      <c r="H22" s="34"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35"/>
-      <c r="K22" s="35"/>
-      <c r="L22" s="39"/>
-    </row>
-    <row r="23" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="53">
+        <v>12</v>
+      </c>
+      <c r="C22" s="52" t="s">
+        <v>80</v>
+      </c>
+      <c r="D22" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="F22" s="36" t="s">
+        <v>53</v>
+      </c>
+      <c r="G22" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="H22" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="I22" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="J22" s="37" t="s">
+        <v>53</v>
+      </c>
+      <c r="K22" s="37">
+        <v>1</v>
+      </c>
+      <c r="L22" s="36">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="M22" s="67" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="24"/>
-      <c r="C23" s="46"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="60"/>
-      <c r="K23" s="60"/>
-      <c r="L23" s="61"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="45"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="34"/>
+      <c r="G23" s="35"/>
+      <c r="H23" s="34"/>
+      <c r="I23" s="35"/>
+      <c r="J23" s="35"/>
+      <c r="K23" s="35"/>
+      <c r="L23" s="35"/>
+      <c r="M23" s="39"/>
+    </row>
+    <row r="24" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="46"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="60"/>
+      <c r="K24" s="60"/>
+      <c r="L24" s="60"/>
+      <c r="M24" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="J1:L1"/>
-    <mergeCell ref="L3:L8"/>
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="M3:M8"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="M22" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>